<commit_message>
Clear company name + Name Lookup table
</commit_message>
<xml_diff>
--- a/output/compagnies_found.xlsx
+++ b/output/compagnies_found.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B133"/>
+  <dimension ref="A1:B166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -719,1306 +719,1702 @@
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">bumitama agri </t>
+          <t xml:space="preserve">everchina intl holdings  </t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">bumitama agri </t>
+          <t xml:space="preserve">everchina intl holdings  </t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">scales  </t>
+          <t xml:space="preserve">bumitama agri </t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">scales  </t>
+          <t xml:space="preserve">bumitama agri </t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">kaveri seed  </t>
+          <t xml:space="preserve">eagle high plantations  </t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">kaveri seed  </t>
+          <t xml:space="preserve">eagle high plantations  </t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>slc agricola sa</t>
+          <t xml:space="preserve">sawit sumbermas sarana  </t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>slc agricola sa</t>
+          <t xml:space="preserve">sawit sumbermas sarana  </t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>pyxus international inc</t>
+          <t xml:space="preserve">al jouf agricultural development  </t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>pyxus international inc</t>
+          <t xml:space="preserve">al jouf agricultural development  </t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">limoneira </t>
+          <t xml:space="preserve">scales  </t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">limoneira </t>
+          <t xml:space="preserve">scales  </t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>adecoagro sa</t>
+          <t xml:space="preserve">inti agri resources  </t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>adecoagro sa</t>
+          <t xml:space="preserve">inti agri resources  </t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">inghams group </t>
+          <t xml:space="preserve">kaveri seed  </t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">inghams group </t>
+          <t xml:space="preserve">kaveri seed  </t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>mhp se</t>
+          <t xml:space="preserve">hap seng plantations holdings </t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>mhp se</t>
+          <t xml:space="preserve">hap seng plantations holdings </t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">select harvests </t>
+          <t xml:space="preserve">boustead plantations </t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">select harvests </t>
+          <t xml:space="preserve">boustead plantations </t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">oceanus group </t>
+          <t xml:space="preserve">genting plantations </t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">oceanus group </t>
+          <t xml:space="preserve">genting plantations </t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">heritage foods </t>
+          <t>slc agricola sa</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">heritage foods </t>
+          <t>slc agricola sa</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">costa group holdings </t>
+          <t>pyxus international inc</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">costa group holdings </t>
+          <t>pyxus international inc</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>scandi standard ab (publ)</t>
+          <t xml:space="preserve">kim loong resources </t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>scandi standard ab (publ)</t>
+          <t xml:space="preserve">kim loong resources </t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">china shengmu organic milk </t>
+          <t xml:space="preserve">kluang rubber  (malaya) </t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">china shengmu organic milk </t>
+          <t xml:space="preserve">kluang rubber  (malaya) </t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">sanford </t>
+          <t xml:space="preserve">limoneira </t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">sanford </t>
+          <t xml:space="preserve">limoneira </t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">tech-bank food  </t>
+          <t>adecoagro sa</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">tech-bank food  </t>
+          <t>adecoagro sa</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>hortifrut sa</t>
+          <t xml:space="preserve">inghams group </t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>hortifrut sa</t>
+          <t xml:space="preserve">inghams group </t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">china modern dairy holdings </t>
+          <t>mhp se</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">china modern dairy holdings </t>
+          <t>mhp se</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">yuan long ping high-tech agriculture  </t>
+          <t xml:space="preserve">select harvests </t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">yuan long ping high-tech agriculture  </t>
+          <t xml:space="preserve">select harvests </t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">cofco joycome foods </t>
+          <t xml:space="preserve">oceanus group </t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">cofco joycome foods </t>
+          <t xml:space="preserve">oceanus group </t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>sipef nv</t>
+          <t xml:space="preserve">ioi  </t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>sipef nv</t>
+          <t xml:space="preserve">ioi  </t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">muyuan foods  </t>
+          <t xml:space="preserve">heritage foods </t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">muyuan foods  </t>
+          <t xml:space="preserve">heritage foods </t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>sapmer sa</t>
+          <t xml:space="preserve">costa group holdings </t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>sapmer sa</t>
+          <t xml:space="preserve">costa group holdings </t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">hokuryo  </t>
+          <t>scandi standard ab (publ)</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t xml:space="preserve">hokuryo  </t>
+          <t>scandi standard ab (publ)</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>kws saat se &amp;  kgaa</t>
+          <t xml:space="preserve">china shengmu organic milk </t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>kws saat se &amp;  kgaa</t>
+          <t xml:space="preserve">china shengmu organic milk </t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ros agro </t>
+          <t xml:space="preserve">bahvest resources </t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t xml:space="preserve">ros agro </t>
+          <t xml:space="preserve">bahvest resources </t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">yuanshengtai dairy farm </t>
+          <t xml:space="preserve">sanford </t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t xml:space="preserve">yuanshengtai dairy farm </t>
+          <t xml:space="preserve">sanford </t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">shandong minhe animal husbandry  </t>
+          <t xml:space="preserve">hunan new wellful  </t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t xml:space="preserve">shandong minhe animal husbandry  </t>
+          <t xml:space="preserve">hunan new wellful  </t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>p/f bakkafrost</t>
+          <t xml:space="preserve">pengdu agriculture &amp; animal husbandry  </t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>p/f bakkafrost</t>
+          <t xml:space="preserve">pengdu agriculture &amp; animal husbandry  </t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">origin enterprises </t>
+          <t xml:space="preserve">techbank food  </t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t xml:space="preserve">origin enterprises </t>
+          <t xml:space="preserve">techbank food  </t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">heilongjiang agriculture  </t>
+          <t>hortifrut sa</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t xml:space="preserve">heilongjiang agriculture  </t>
+          <t>hortifrut sa</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">zoneco group  </t>
+          <t xml:space="preserve">a2 milk  </t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t xml:space="preserve">zoneco group  </t>
+          <t xml:space="preserve">a2 milk  </t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">shandong yisheng livestock &amp; poultry breeding  </t>
+          <t xml:space="preserve">jiangxi zhengbang technology  </t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t xml:space="preserve">shandong yisheng livestock &amp; poultry breeding  </t>
+          <t xml:space="preserve">jiangxi zhengbang technology  </t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">uie </t>
+          <t xml:space="preserve">al gassim investment holding  </t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t xml:space="preserve">uie </t>
+          <t xml:space="preserve">al gassim investment holding  </t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">anglo-eastern plantations </t>
+          <t xml:space="preserve">china modern dairy holdings </t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t xml:space="preserve">anglo-eastern plantations </t>
+          <t xml:space="preserve">china modern dairy holdings </t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">luoniushan  </t>
+          <t xml:space="preserve">yuan long ping hightech agriculture  </t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t xml:space="preserve">luoniushan  </t>
+          <t xml:space="preserve">yuan long ping hightech agriculture  </t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">shandong xiantan  </t>
+          <t xml:space="preserve">shandong denghai seeds  </t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t xml:space="preserve">shandong xiantan  </t>
+          <t xml:space="preserve">shandong denghai seeds  </t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">synlait milk </t>
+          <t xml:space="preserve">cofco joycome foods </t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t xml:space="preserve">synlait milk </t>
+          <t xml:space="preserve">cofco joycome foods </t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>grieg seafood asa</t>
+          <t>sipef nv</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>grieg seafood asa</t>
+          <t>sipef nv</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">hokuto </t>
+          <t xml:space="preserve">muyuan foods  </t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t xml:space="preserve">hokuto </t>
+          <t xml:space="preserve">muyuan foods  </t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">winall hi-tech seed  </t>
+          <t xml:space="preserve">bakrie sumatera plantations  </t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t xml:space="preserve">winall hi-tech seed  </t>
+          <t xml:space="preserve">bakrie sumatera plantations  </t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>vilmorin &amp; cie sa</t>
+          <t>sapmer sa</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>vilmorin &amp; cie sa</t>
+          <t>sapmer sa</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>agrogeneration sa</t>
+          <t xml:space="preserve">hokuryo  </t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>agrogeneration sa</t>
+          <t xml:space="preserve">hokuryo  </t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>kernel holding sa</t>
+          <t>kws saat se &amp;  kgaa</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>kernel holding sa</t>
+          <t>kws saat se &amp;  kgaa</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">xinjiang sayram modern agriculture  </t>
+          <t xml:space="preserve">far east holdings </t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t xml:space="preserve">xinjiang sayram modern agriculture  </t>
+          <t xml:space="preserve">far east holdings </t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>cal-maine foods inc</t>
+          <t xml:space="preserve">ros agro </t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>cal-maine foods inc</t>
+          <t xml:space="preserve">ros agro </t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">first resources </t>
+          <t xml:space="preserve">yuanshengtai dairy farm </t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t xml:space="preserve">first resources </t>
+          <t xml:space="preserve">yuanshengtai dairy farm </t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">jiangsu yangnong chemical  </t>
+          <t xml:space="preserve">shandong minhe animal husbandry  </t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t xml:space="preserve">jiangsu yangnong chemical  </t>
+          <t xml:space="preserve">shandong minhe animal husbandry  </t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">kingenta ecological engineering group  </t>
+          <t>p/f bakkafrost</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t xml:space="preserve">kingenta ecological engineering group  </t>
+          <t>p/f bakkafrost</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">dawood hercules  </t>
+          <t>gruppa cherkizovo pao</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t xml:space="preserve">dawood hercules  </t>
+          <t>gruppa cherkizovo pao</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">hubei yihua chemical industry  </t>
+          <t xml:space="preserve">origin enterprises </t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t xml:space="preserve">hubei yihua chemical industry  </t>
+          <t xml:space="preserve">origin enterprises </t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">yonfer agricultural technology  </t>
+          <t xml:space="preserve">heilongjiang agriculture  </t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t xml:space="preserve">yonfer agricultural technology  </t>
+          <t xml:space="preserve">heilongjiang agriculture  </t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">sharda cropchem </t>
+          <t xml:space="preserve">zoneco group  </t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t xml:space="preserve">sharda cropchem </t>
+          <t xml:space="preserve">zoneco group  </t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">engro fertilizers </t>
+          <t xml:space="preserve">shandong yisheng livestock &amp; poultry breeding  </t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t xml:space="preserve">engro fertilizers </t>
+          <t xml:space="preserve">shandong yisheng livestock &amp; poultry breeding  </t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">china bozza development holdings </t>
+          <t xml:space="preserve">united malacca </t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t xml:space="preserve">china bozza development holdings </t>
+          <t xml:space="preserve">united malacca </t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">acadian timber </t>
+          <t xml:space="preserve">uie </t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t xml:space="preserve">acadian timber </t>
+          <t xml:space="preserve">uie </t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">rallis india </t>
+          <t xml:space="preserve">angloeastern plantations </t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t xml:space="preserve">rallis india </t>
+          <t xml:space="preserve">angloeastern plantations </t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">agro-kanesho  </t>
+          <t xml:space="preserve">luoniushan  </t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t xml:space="preserve">agro-kanesho  </t>
+          <t xml:space="preserve">luoniushan  </t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">taiwan fertilizer  </t>
+          <t xml:space="preserve">shandong xiantan  </t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t xml:space="preserve">taiwan fertilizer  </t>
+          <t xml:space="preserve">shandong xiantan  </t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">china xlx fertiliser </t>
+          <t xml:space="preserve">synlait milk </t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t xml:space="preserve">china xlx fertiliser </t>
+          <t xml:space="preserve">synlait milk </t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">rashtriya chemicals and fertilizers </t>
+          <t>grieg seafood asa</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t xml:space="preserve">rashtriya chemicals and fertilizers </t>
+          <t>grieg seafood asa</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">shenzhen noposion crop science  </t>
+          <t xml:space="preserve">hokuto </t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t xml:space="preserve">shenzhen noposion crop science  </t>
+          <t xml:space="preserve">hokuto </t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>grupa azoty sa</t>
+          <t xml:space="preserve">saudi fisheries  </t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>grupa azoty sa</t>
+          <t xml:space="preserve">saudi fisheries  </t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">shenzhen batian ecotypic engineering  </t>
+          <t xml:space="preserve">winall hitech seed  </t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t xml:space="preserve">shenzhen batian ecotypic engineering  </t>
+          <t xml:space="preserve">winall hitech seed  </t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ch biotech r&amp;d  </t>
+          <t xml:space="preserve">tsh resources </t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t xml:space="preserve">ch biotech r&amp;d  </t>
+          <t xml:space="preserve">tsh resources </t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">china bluechemical </t>
+          <t>vilmorin &amp; cie sa</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t xml:space="preserve">china bluechemical </t>
+          <t>vilmorin &amp; cie sa</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">katakura &amp; -op agri </t>
+          <t>agrogeneration sa</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t xml:space="preserve">katakura &amp; -op agri </t>
+          <t>agrogeneration sa</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">astec lifesciences </t>
+          <t xml:space="preserve">tabuk agricultural development  </t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t xml:space="preserve">astec lifesciences </t>
+          <t xml:space="preserve">tabuk agricultural development  </t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">oat agrio  </t>
+          <t xml:space="preserve">sarawak oil palms </t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t xml:space="preserve">oat agrio  </t>
+          <t xml:space="preserve">sarawak oil palms </t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">chengdu wintrue holding  </t>
+          <t>kernel holding sa</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t xml:space="preserve">chengdu wintrue holding  </t>
+          <t>kernel holding sa</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">american vanguard </t>
+          <t xml:space="preserve">xinjiang sayram modern agriculture  </t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t xml:space="preserve">american vanguard </t>
+          <t xml:space="preserve">xinjiang sayram modern agriculture  </t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">fatima fertilizer  </t>
+          <t>calmaine foods inc</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t xml:space="preserve">fatima fertilizer  </t>
+          <t>calmaine foods inc</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">suli  </t>
+          <t xml:space="preserve">first resources </t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t xml:space="preserve">suli  </t>
+          <t xml:space="preserve">first resources </t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">tianjin teda biomedical engineering  </t>
+          <t xml:space="preserve">fgv holdings </t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t xml:space="preserve">tianjin teda biomedical engineering  </t>
+          <t xml:space="preserve">fgv holdings </t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">nufarm </t>
+          <t xml:space="preserve">jiangsu yangnong chemical  </t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t xml:space="preserve">nufarm </t>
+          <t xml:space="preserve">jiangsu yangnong chemical  </t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">bharat rasayan </t>
+          <t xml:space="preserve">kingenta ecological engineering group  </t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t xml:space="preserve">bharat rasayan </t>
+          <t xml:space="preserve">kingenta ecological engineering group  </t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>oci nv</t>
+          <t xml:space="preserve">dawood hercules  </t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>oci nv</t>
+          <t xml:space="preserve">dawood hercules  </t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">anhui guangxin agrochemical  </t>
+          <t xml:space="preserve">hubei yihua chemical industry  </t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t xml:space="preserve">anhui guangxin agrochemical  </t>
+          <t xml:space="preserve">hubei yihua chemical industry  </t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>eucatex sa industria e comercio</t>
+          <t xml:space="preserve">yonfer agricultural technology  </t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>eucatex sa industria e comercio</t>
+          <t xml:space="preserve">yonfer agricultural technology  </t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>western forest products inc</t>
+          <t xml:space="preserve">sharda cropchem </t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>western forest products inc</t>
+          <t xml:space="preserve">sharda cropchem </t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">jiangsu yabang dyestuff  </t>
+          <t>misr fertilizers production  sae</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t xml:space="preserve">jiangsu yabang dyestuff  </t>
+          <t>misr fertilizers production  sae</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">omnia holdings </t>
+          <t xml:space="preserve">engro fertilizers </t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t xml:space="preserve">omnia holdings </t>
+          <t xml:space="preserve">engro fertilizers </t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>lsb industries inc</t>
+          <t xml:space="preserve">w t k holdings </t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>lsb industries inc</t>
+          <t xml:space="preserve">w t k holdings </t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>hawkins inc</t>
+          <t xml:space="preserve">china bozza development holdings </t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>hawkins inc</t>
+          <t xml:space="preserve">china bozza development holdings </t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">meghmani organics </t>
+          <t xml:space="preserve">acadian timber </t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t xml:space="preserve">meghmani organics </t>
+          <t xml:space="preserve">acadian timber </t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>exel industries sa</t>
+          <t xml:space="preserve">rallis india </t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>exel industries sa</t>
+          <t xml:space="preserve">rallis india </t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t>ag growth international inc</t>
+          <t xml:space="preserve">stanley agricultural group  </t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>ag growth international inc</t>
+          <t xml:space="preserve">stanley agricultural group  </t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">nippon soda  </t>
+          <t xml:space="preserve">agrokanesho  </t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t xml:space="preserve">nippon soda  </t>
+          <t xml:space="preserve">agrokanesho  </t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">nihon nohyaku  </t>
+          <t xml:space="preserve">taiwan fertilizer  </t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t xml:space="preserve">nihon nohyaku  </t>
+          <t xml:space="preserve">taiwan fertilizer  </t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">nissan chemical </t>
+          <t xml:space="preserve">china xlx fertiliser </t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t xml:space="preserve">nissan chemical </t>
+          <t xml:space="preserve">china xlx fertiliser </t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">kumiai chemical industry  </t>
+          <t xml:space="preserve">rashtriya chemicals and fertilizers </t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t xml:space="preserve">kumiai chemical industry  </t>
+          <t xml:space="preserve">rashtriya chemicals and fertilizers </t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">hokko chemical industry  </t>
+          <t xml:space="preserve">shenzhen noposion crop science  </t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t xml:space="preserve">hokko chemical industry  </t>
+          <t xml:space="preserve">shenzhen noposion crop science  </t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">fumakilla </t>
+          <t>grupa azoty sa</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t xml:space="preserve">fumakilla </t>
+          <t>grupa azoty sa</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">kal group </t>
+          <t xml:space="preserve">shenzhen batian ecotypic engineering  </t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t xml:space="preserve">kal group </t>
+          <t xml:space="preserve">shenzhen batian ecotypic engineering  </t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">sumitomo chemical india </t>
+          <t xml:space="preserve">ch biotech r&amp;d  </t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t xml:space="preserve">sumitomo chemical india </t>
+          <t xml:space="preserve">ch biotech r&amp;d  </t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">dalian bio-chem  </t>
+          <t xml:space="preserve">china bluechemical </t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t xml:space="preserve">dalian bio-chem  </t>
+          <t xml:space="preserve">china bluechemical </t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">sea harvest group </t>
+          <t xml:space="preserve">katakura &amp; coop agri </t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t xml:space="preserve">sea harvest group </t>
+          <t xml:space="preserve">katakura &amp; coop agri </t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">jiangsu lihua animal husbandry  </t>
+          <t xml:space="preserve">astec lifesciences </t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t xml:space="preserve">jiangsu lihua animal husbandry  </t>
+          <t xml:space="preserve">astec lifesciences </t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">adama </t>
+          <t xml:space="preserve">oat agrio  </t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t xml:space="preserve">adama </t>
+          <t xml:space="preserve">oat agrio  </t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">china fishery group </t>
+          <t xml:space="preserve">chengdu wintrue holding  </t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t xml:space="preserve">china fishery group </t>
+          <t xml:space="preserve">chengdu wintrue holding  </t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">heranba industries </t>
+          <t xml:space="preserve">american vanguard </t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t xml:space="preserve">heranba industries </t>
+          <t xml:space="preserve">american vanguard </t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>atlantic sapphire asa</t>
+          <t xml:space="preserve">fatima fertilizer  </t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>atlantic sapphire asa</t>
+          <t xml:space="preserve">fatima fertilizer  </t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">guizhou chanhen chemical </t>
+          <t xml:space="preserve">suli  </t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t xml:space="preserve">guizhou chanhen chemical </t>
+          <t xml:space="preserve">suli  </t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>salmones camanchaca sa</t>
+          <t xml:space="preserve">tianjin teda biomedical engineering  </t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>salmones camanchaca sa</t>
+          <t xml:space="preserve">tianjin teda biomedical engineering  </t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>appharvest inc</t>
+          <t xml:space="preserve">nufarm </t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>appharvest inc</t>
+          <t xml:space="preserve">nufarm </t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>vittia sa</t>
+          <t xml:space="preserve">bharat rasayan </t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>vittia sa</t>
+          <t xml:space="preserve">bharat rasayan </t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">agrify </t>
+          <t>oci nv</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t xml:space="preserve">agrify </t>
+          <t>oci nv</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">anhui guangxin agrochemical  </t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">anhui guangxin agrochemical  </t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="1" t="inlineStr">
+        <is>
+          <t>eucatex sa industria e comercio</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>eucatex sa industria e comercio</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">jaya tiasa holdings </t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">jaya tiasa holdings </t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="1" t="inlineStr">
+        <is>
+          <t>western forest products inc</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>western forest products inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">jiangsu yabang dyestuff  </t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">jiangsu yabang dyestuff  </t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">omnia holdings </t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">omnia holdings </t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="1" t="inlineStr">
+        <is>
+          <t>lsb industries inc</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>lsb industries inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="1" t="inlineStr">
+        <is>
+          <t>hawkins inc</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>hawkins inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">meghmani organics </t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">meghmani organics </t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="1" t="inlineStr">
+        <is>
+          <t>exel industries sa</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>exel industries sa</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="1" t="inlineStr">
+        <is>
+          <t>ag growth international inc</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>ag growth international inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nippon soda  </t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nippon soda  </t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nihon nohyaku  </t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nihon nohyaku  </t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nissan chemical </t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t xml:space="preserve">nissan chemical </t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kumiai chemical industry  </t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kumiai chemical industry  </t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hokko chemical industry  </t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hokko chemical industry  </t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fumakilla </t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fumakilla </t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kal group </t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kal group </t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sumitomo chemical india </t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sumitomo chemical india </t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dalian biochem  </t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dalian biochem  </t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sea harvest group </t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sea harvest group </t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">jiangsu lihua animal husbandry  </t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t xml:space="preserve">jiangsu lihua animal husbandry  </t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">adama </t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t xml:space="preserve">adama </t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">china fishery group </t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t xml:space="preserve">china fishery group </t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">heranba industries </t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t xml:space="preserve">heranba industries </t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="1" t="inlineStr">
+        <is>
+          <t>atlantic sapphire asa</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>atlantic sapphire asa</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">leong hup international </t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t xml:space="preserve">leong hup international </t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">guizhou chanhen chemical </t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">guizhou chanhen chemical </t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="1" t="inlineStr">
+        <is>
+          <t>salmones camanchaca sa</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>salmones camanchaca sa</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hextar global </t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hextar global </t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="1" t="inlineStr">
+        <is>
+          <t>appharvest inc</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>appharvest inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="1" t="inlineStr">
+        <is>
+          <t>vittia sa</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>vittia sa</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">agrify </t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t xml:space="preserve">agrify </t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">cheerwin group </t>
         </is>
       </c>
-      <c r="B133" t="inlineStr">
+      <c r="B166" t="inlineStr">
         <is>
           <t xml:space="preserve">cheerwin group </t>
         </is>

</xml_diff>

<commit_message>
Add Refinitiv controls var 2004&2022
</commit_message>
<xml_diff>
--- a/output/compagnies_found.xlsx
+++ b/output/compagnies_found.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B166"/>
+  <dimension ref="A1:B164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1511,910 +1511,886 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>vilmorin &amp; cie sa</t>
+          <t>agrogeneration sa</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>vilmorin &amp; cie sa</t>
+          <t>agrogeneration sa</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>agrogeneration sa</t>
+          <t xml:space="preserve">tabuk agricultural development  </t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>agrogeneration sa</t>
+          <t xml:space="preserve">tabuk agricultural development  </t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">tabuk agricultural development  </t>
+          <t xml:space="preserve">sarawak oil palms </t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t xml:space="preserve">tabuk agricultural development  </t>
+          <t xml:space="preserve">sarawak oil palms </t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">sarawak oil palms </t>
+          <t>kernel holding sa</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t xml:space="preserve">sarawak oil palms </t>
+          <t>kernel holding sa</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>kernel holding sa</t>
+          <t xml:space="preserve">xinjiang sayram modern agriculture  </t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>kernel holding sa</t>
+          <t xml:space="preserve">xinjiang sayram modern agriculture  </t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">xinjiang sayram modern agriculture  </t>
+          <t>calmaine foods inc</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t xml:space="preserve">xinjiang sayram modern agriculture  </t>
+          <t>calmaine foods inc</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>calmaine foods inc</t>
+          <t xml:space="preserve">first resources </t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>calmaine foods inc</t>
+          <t xml:space="preserve">first resources </t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">first resources </t>
+          <t xml:space="preserve">fgv holdings </t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t xml:space="preserve">first resources </t>
+          <t xml:space="preserve">fgv holdings </t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">fgv holdings </t>
+          <t xml:space="preserve">jiangsu yangnong chemical  </t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t xml:space="preserve">fgv holdings </t>
+          <t xml:space="preserve">jiangsu yangnong chemical  </t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">jiangsu yangnong chemical  </t>
+          <t xml:space="preserve">kingenta ecological engineering group  </t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t xml:space="preserve">jiangsu yangnong chemical  </t>
+          <t xml:space="preserve">kingenta ecological engineering group  </t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">kingenta ecological engineering group  </t>
+          <t xml:space="preserve">dawood hercules  </t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t xml:space="preserve">kingenta ecological engineering group  </t>
+          <t xml:space="preserve">dawood hercules  </t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">dawood hercules  </t>
+          <t xml:space="preserve">hubei yihua chemical industry  </t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t xml:space="preserve">dawood hercules  </t>
+          <t xml:space="preserve">hubei yihua chemical industry  </t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">hubei yihua chemical industry  </t>
+          <t xml:space="preserve">yonfer agricultural technology  </t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t xml:space="preserve">hubei yihua chemical industry  </t>
+          <t xml:space="preserve">yonfer agricultural technology  </t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">yonfer agricultural technology  </t>
+          <t xml:space="preserve">sharda cropchem </t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t xml:space="preserve">yonfer agricultural technology  </t>
+          <t xml:space="preserve">sharda cropchem </t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">sharda cropchem </t>
+          <t>misr fertilizers production  sae</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t xml:space="preserve">sharda cropchem </t>
+          <t>misr fertilizers production  sae</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>misr fertilizers production  sae</t>
+          <t xml:space="preserve">engro fertilizers </t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>misr fertilizers production  sae</t>
+          <t xml:space="preserve">engro fertilizers </t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">engro fertilizers </t>
+          <t xml:space="preserve">w t k holdings </t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t xml:space="preserve">engro fertilizers </t>
+          <t xml:space="preserve">w t k holdings </t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">w t k holdings </t>
+          <t xml:space="preserve">china bozza development holdings </t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t xml:space="preserve">w t k holdings </t>
+          <t xml:space="preserve">china bozza development holdings </t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">china bozza development holdings </t>
+          <t xml:space="preserve">acadian timber </t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t xml:space="preserve">china bozza development holdings </t>
+          <t xml:space="preserve">acadian timber </t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">acadian timber </t>
+          <t xml:space="preserve">rallis india </t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t xml:space="preserve">acadian timber </t>
+          <t xml:space="preserve">rallis india </t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">rallis india </t>
+          <t xml:space="preserve">agrokanesho  </t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t xml:space="preserve">rallis india </t>
+          <t xml:space="preserve">agrokanesho  </t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">stanley agricultural group  </t>
+          <t xml:space="preserve">taiwan fertilizer  </t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t xml:space="preserve">stanley agricultural group  </t>
+          <t xml:space="preserve">taiwan fertilizer  </t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">agrokanesho  </t>
+          <t xml:space="preserve">china xlx fertiliser </t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t xml:space="preserve">agrokanesho  </t>
+          <t xml:space="preserve">china xlx fertiliser </t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">taiwan fertilizer  </t>
+          <t xml:space="preserve">rashtriya chemicals and fertilizers </t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t xml:space="preserve">taiwan fertilizer  </t>
+          <t xml:space="preserve">rashtriya chemicals and fertilizers </t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">china xlx fertiliser </t>
+          <t xml:space="preserve">shenzhen noposion crop science  </t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t xml:space="preserve">china xlx fertiliser </t>
+          <t xml:space="preserve">shenzhen noposion crop science  </t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">rashtriya chemicals and fertilizers </t>
+          <t>grupa azoty sa</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t xml:space="preserve">rashtriya chemicals and fertilizers </t>
+          <t>grupa azoty sa</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">shenzhen noposion crop science  </t>
+          <t xml:space="preserve">shenzhen batian ecotypic engineering  </t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t xml:space="preserve">shenzhen noposion crop science  </t>
+          <t xml:space="preserve">shenzhen batian ecotypic engineering  </t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>grupa azoty sa</t>
+          <t xml:space="preserve">ch biotech r&amp;d  </t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>grupa azoty sa</t>
+          <t xml:space="preserve">ch biotech r&amp;d  </t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">shenzhen batian ecotypic engineering  </t>
+          <t xml:space="preserve">china bluechemical </t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t xml:space="preserve">shenzhen batian ecotypic engineering  </t>
+          <t xml:space="preserve">china bluechemical </t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ch biotech r&amp;d  </t>
+          <t xml:space="preserve">katakura &amp; coop agri </t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t xml:space="preserve">ch biotech r&amp;d  </t>
+          <t xml:space="preserve">katakura &amp; coop agri </t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">china bluechemical </t>
+          <t xml:space="preserve">astec lifesciences </t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t xml:space="preserve">china bluechemical </t>
+          <t xml:space="preserve">astec lifesciences </t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">katakura &amp; coop agri </t>
+          <t xml:space="preserve">oat agrio  </t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t xml:space="preserve">katakura &amp; coop agri </t>
+          <t xml:space="preserve">oat agrio  </t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">astec lifesciences </t>
+          <t xml:space="preserve">chengdu wintrue holding  </t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t xml:space="preserve">astec lifesciences </t>
+          <t xml:space="preserve">chengdu wintrue holding  </t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">oat agrio  </t>
+          <t xml:space="preserve">american vanguard </t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t xml:space="preserve">oat agrio  </t>
+          <t xml:space="preserve">american vanguard </t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">chengdu wintrue holding  </t>
+          <t xml:space="preserve">fatima fertilizer  </t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t xml:space="preserve">chengdu wintrue holding  </t>
+          <t xml:space="preserve">fatima fertilizer  </t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">american vanguard </t>
+          <t xml:space="preserve">suli  </t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t xml:space="preserve">american vanguard </t>
+          <t xml:space="preserve">suli  </t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">fatima fertilizer  </t>
+          <t xml:space="preserve">tianjin teda biomedical engineering  </t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t xml:space="preserve">fatima fertilizer  </t>
+          <t xml:space="preserve">tianjin teda biomedical engineering  </t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">suli  </t>
+          <t xml:space="preserve">nufarm </t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t xml:space="preserve">suli  </t>
+          <t xml:space="preserve">nufarm </t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">tianjin teda biomedical engineering  </t>
+          <t xml:space="preserve">bharat rasayan </t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t xml:space="preserve">tianjin teda biomedical engineering  </t>
+          <t xml:space="preserve">bharat rasayan </t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">nufarm </t>
+          <t>oci nv</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t xml:space="preserve">nufarm </t>
+          <t>oci nv</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">bharat rasayan </t>
+          <t xml:space="preserve">anhui guangxin agrochemical  </t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t xml:space="preserve">bharat rasayan </t>
+          <t xml:space="preserve">anhui guangxin agrochemical  </t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>oci nv</t>
+          <t>eucatex sa industria e comercio</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>oci nv</t>
+          <t>eucatex sa industria e comercio</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">anhui guangxin agrochemical  </t>
+          <t xml:space="preserve">jaya tiasa holdings </t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t xml:space="preserve">anhui guangxin agrochemical  </t>
+          <t xml:space="preserve">jaya tiasa holdings </t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>eucatex sa industria e comercio</t>
+          <t>western forest products inc</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>eucatex sa industria e comercio</t>
+          <t>western forest products inc</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">jaya tiasa holdings </t>
+          <t xml:space="preserve">jiangsu yabang dyestuff  </t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t xml:space="preserve">jaya tiasa holdings </t>
+          <t xml:space="preserve">jiangsu yabang dyestuff  </t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>western forest products inc</t>
+          <t xml:space="preserve">omnia holdings </t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>western forest products inc</t>
+          <t xml:space="preserve">omnia holdings </t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">jiangsu yabang dyestuff  </t>
+          <t>lsb industries inc</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t xml:space="preserve">jiangsu yabang dyestuff  </t>
+          <t>lsb industries inc</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">omnia holdings </t>
+          <t>hawkins inc</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t xml:space="preserve">omnia holdings </t>
+          <t>hawkins inc</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>lsb industries inc</t>
+          <t xml:space="preserve">meghmani organics </t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>lsb industries inc</t>
+          <t xml:space="preserve">meghmani organics </t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>hawkins inc</t>
+          <t>exel industries sa</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>hawkins inc</t>
+          <t>exel industries sa</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">meghmani organics </t>
+          <t>ag growth international inc</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t xml:space="preserve">meghmani organics </t>
+          <t>ag growth international inc</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="1" t="inlineStr">
         <is>
-          <t>exel industries sa</t>
+          <t xml:space="preserve">nippon soda  </t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>exel industries sa</t>
+          <t xml:space="preserve">nippon soda  </t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>ag growth international inc</t>
+          <t xml:space="preserve">nihon nohyaku  </t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>ag growth international inc</t>
+          <t xml:space="preserve">nihon nohyaku  </t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">nippon soda  </t>
+          <t xml:space="preserve">nissan chemical </t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t xml:space="preserve">nippon soda  </t>
+          <t xml:space="preserve">nissan chemical </t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">nihon nohyaku  </t>
+          <t xml:space="preserve">kumiai chemical industry  </t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t xml:space="preserve">nihon nohyaku  </t>
+          <t xml:space="preserve">kumiai chemical industry  </t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">nissan chemical </t>
+          <t xml:space="preserve">hokko chemical industry  </t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t xml:space="preserve">nissan chemical </t>
+          <t xml:space="preserve">hokko chemical industry  </t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">kumiai chemical industry  </t>
+          <t xml:space="preserve">fumakilla </t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t xml:space="preserve">kumiai chemical industry  </t>
+          <t xml:space="preserve">fumakilla </t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">hokko chemical industry  </t>
+          <t xml:space="preserve">kal group </t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t xml:space="preserve">hokko chemical industry  </t>
+          <t xml:space="preserve">kal group </t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">fumakilla </t>
+          <t xml:space="preserve">sumitomo chemical india </t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t xml:space="preserve">fumakilla </t>
+          <t xml:space="preserve">sumitomo chemical india </t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">kal group </t>
+          <t xml:space="preserve">dalian biochem  </t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t xml:space="preserve">kal group </t>
+          <t xml:space="preserve">dalian biochem  </t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">sumitomo chemical india </t>
+          <t xml:space="preserve">sea harvest group </t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t xml:space="preserve">sumitomo chemical india </t>
+          <t xml:space="preserve">sea harvest group </t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">dalian biochem  </t>
+          <t xml:space="preserve">jiangsu lihua animal husbandry  </t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t xml:space="preserve">dalian biochem  </t>
+          <t xml:space="preserve">jiangsu lihua animal husbandry  </t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">sea harvest group </t>
+          <t xml:space="preserve">adama </t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t xml:space="preserve">sea harvest group </t>
+          <t xml:space="preserve">adama </t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">jiangsu lihua animal husbandry  </t>
+          <t xml:space="preserve">china fishery group </t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t xml:space="preserve">jiangsu lihua animal husbandry  </t>
+          <t xml:space="preserve">china fishery group </t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">adama </t>
+          <t xml:space="preserve">heranba industries </t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t xml:space="preserve">adama </t>
+          <t xml:space="preserve">heranba industries </t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">china fishery group </t>
+          <t>atlantic sapphire asa</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t xml:space="preserve">china fishery group </t>
+          <t>atlantic sapphire asa</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">heranba industries </t>
+          <t xml:space="preserve">leong hup international </t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t xml:space="preserve">heranba industries </t>
+          <t xml:space="preserve">leong hup international </t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>atlantic sapphire asa</t>
+          <t xml:space="preserve">guizhou chanhen chemical </t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>atlantic sapphire asa</t>
+          <t xml:space="preserve">guizhou chanhen chemical </t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">leong hup international </t>
+          <t>salmones camanchaca sa</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t xml:space="preserve">leong hup international </t>
+          <t>salmones camanchaca sa</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">guizhou chanhen chemical </t>
+          <t xml:space="preserve">hextar global </t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t xml:space="preserve">guizhou chanhen chemical </t>
+          <t xml:space="preserve">hextar global </t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>salmones camanchaca sa</t>
+          <t>appharvest inc</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>salmones camanchaca sa</t>
+          <t>appharvest inc</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">hextar global </t>
+          <t>vittia sa</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t xml:space="preserve">hextar global </t>
+          <t>vittia sa</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>appharvest inc</t>
+          <t xml:space="preserve">agrify </t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>appharvest inc</t>
+          <t xml:space="preserve">agrify </t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>vittia sa</t>
+          <t xml:space="preserve">cheerwin group </t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
-        <is>
-          <t>vittia sa</t>
-        </is>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">agrify </t>
-        </is>
-      </c>
-      <c r="B165" t="inlineStr">
-        <is>
-          <t xml:space="preserve">agrify </t>
-        </is>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">cheerwin group </t>
-        </is>
-      </c>
-      <c r="B166" t="inlineStr">
         <is>
           <t xml:space="preserve">cheerwin group </t>
         </is>

</xml_diff>